<commit_message>
feat(import): adopt PM's updated form layout - Project Superintendent (migration 0007), combined Foreman/Lead, 6 system slots; fix(ci): RESEND secret conditional via job-level env (workflow failed to parse with secrets in step if)
</commit_message>
<xml_diff>
--- a/web/public/templates/3DTSI-Project-Form.xlsx
+++ b/web/public/templates/3DTSI-Project-Form.xlsx
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="46">
   <si>
     <t>3DTSI PROJECT SETUP FORM</t>
   </si>
@@ -118,10 +118,10 @@
     <t>Project Manager</t>
   </si>
   <si>
-    <t>Project Foreman</t>
-  </si>
-  <si>
-    <t>Project Lead</t>
+    <t>Project Superintendent</t>
+  </si>
+  <si>
+    <t>Project Foreman / Lead</t>
   </si>
   <si>
     <t>Project System #1</t>
@@ -137,6 +137,9 @@
   </si>
   <si>
     <t>Project System #5</t>
+  </si>
+  <si>
+    <t>Project System #6</t>
   </si>
   <si>
     <t>Systems</t>
@@ -655,7 +658,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -778,13 +781,19 @@
       </c>
       <c r="B19" s="5"/>
     </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20" s="5"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Pick from the list" error="Choose a value from the dropdown (see Reference sheet)." sqref="B15:B19">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Pick from the list" error="Choose a value from the dropdown (see Reference sheet)." sqref="B15:B20">
       <formula1>Reference!$A$2:$A$12</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Pick from the list" error="Choose a value from the dropdown (see Reference sheet)." sqref="B8">
@@ -812,104 +821,104 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>